<commit_message>
Alinea los cuadernos 1 y 4 a 7 con la muestra de 108 y un solo calendario, y agrega la plantilla de la sesión 8.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/instrumentos/sesion-01/Sesion 1.xlsx
+++ b/instrumentos/sesion-01/Sesion 1.xlsx
@@ -8553,7 +8553,7 @@
       </c>
       <c r="C11" s="30" t="inlineStr">
         <is>
-          <t>Aplicación multiplataforma de búsqueda semántica conversacional: uso libre de la aplicación durante 7 días, con al menos 3 sesiones de consulta verificadas con la telemetría, del 18/11/2026 al 24/11/2026 (PDT §3.3).</t>
+          <t>Aplicación multiplataforma de búsqueda semántica conversacional: uso libre de la aplicación durante 7 días, con al menos 3 sesiones de consulta verificadas con la telemetría, del 27/10/2026 al 02/11/2026 (PDT §3.3).</t>
         </is>
       </c>
       <c r="D11" s="73" t="inlineStr">
@@ -8740,9 +8740,9 @@
       </c>
       <c r="C15" s="30" t="inlineStr">
         <is>
-          <t>Pretest: 11/11/2026 al 16/11/2026 (hoja 3, actividad 9).
-Intervención: 18/11/2026 al 24/11/2026 (7 días, actividad 11).
-Postest: 25/11/2026 al 30/11/2026 (actividad 12), con holgura del 01 al 06/12/2026.
+          <t>Pretest: 20/10/2026 al 25/10/2026 (hoja 3, actividad 9).
+Intervención: 27/10/2026 al 02/11/2026 (7 días, actividad 11).
+Postest: 03/11/2026 al 08/11/2026 (actividad 12), con holgura del 09 al 15/11/2026.
 Justificación: 7 días permiten al menos 3 sesiones de uso real sin alargar la exposición a eventos externos ni la pérdida de participantes; todo termina antes del vencimiento de la autorización (diciembre de 2026) y de la retención de las noticias de las tareas.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Corre el calendario de campo ocho días atrás y consolida la base simulada de la sesión 8.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/instrumentos/sesion-01/Sesion 1.xlsx
+++ b/instrumentos/sesion-01/Sesion 1.xlsx
@@ -8553,7 +8553,7 @@
       </c>
       <c r="C11" s="30" t="inlineStr">
         <is>
-          <t>Aplicación multiplataforma de búsqueda semántica conversacional: uso libre de la aplicación durante 7 días, con al menos 3 sesiones de consulta verificadas con la telemetría, del 27/10/2026 al 02/11/2026 (PDT §3.3).</t>
+          <t>Aplicación multiplataforma de búsqueda semántica conversacional: uso libre de la aplicación durante 7 días, con al menos 3 sesiones de consulta verificadas con la telemetría, del 19/10/2026 al 25/10/2026 (PDT §3.3).</t>
         </is>
       </c>
       <c r="D11" s="73" t="inlineStr">
@@ -8648,7 +8648,7 @@
           <t>1. Cuestionario SUS (10 ítems): juicio de 2 expertos y 1 juez.
 2. Cuestionario de satisfacción de uso adaptado de TAM: juicio de 4 expertos y 2 jueces.
 3. Ficha de registro de tiempos y clics: registro automático, sin validación por juicio.
-V de Aiken ≥ 0.80 por ítem (PDT §3.5.3). Confiabilidad: alfa de Cronbach &gt; 0.70 en un piloto de 20 lectores ajenos a la muestra (PDT §3.5.4). Estado: juicio de expertos programado del 12 al 24/10/2026 y piloto del 02 al 05/11/2026; aún no hay resultados que reportar.</t>
+V de Aiken ≥ 0.80 por ítem (PDT §3.5.3). Confiabilidad: alfa de Cronbach &gt; 0.70 en un piloto de 20 lectores ajenos a la muestra (PDT §3.5.4). Estado: juicio de expertos programado del 12 al 16/10/2026 y piloto del 02 al 28/10/2026; aún no hay resultados que reportar.</t>
         </is>
       </c>
       <c r="D13" s="73" t="inlineStr">
@@ -8740,9 +8740,9 @@
       </c>
       <c r="C15" s="30" t="inlineStr">
         <is>
-          <t>Pretest: 20/10/2026 al 25/10/2026 (hoja 3, actividad 9).
-Intervención: 27/10/2026 al 02/11/2026 (7 días, actividad 11).
-Postest: 03/11/2026 al 08/11/2026 (actividad 12), con holgura del 09 al 15/11/2026.
+          <t>Pretest: 12/10/2026 al 17/10/2026 (hoja 3, actividad 9).
+Intervención: 19/10/2026 al 25/10/2026 (7 días, actividad 11).
+Postest: 26/10/2026 al 31/10/2026 (actividad 12), con holgura del 01 al 07/11/2026.
 Justificación: 7 días permiten al menos 3 sesiones de uso real sin alargar la exposición a eventos externos ni la pérdida de participantes; todo termina antes del vencimiento de la autorización (diciembre de 2026) y de la retención de las noticias de las tareas.</t>
         </is>
       </c>
@@ -15616,10 +15616,10 @@
         </is>
       </c>
       <c r="C7" s="22" t="n">
-        <v>46307</v>
+        <v>46299</v>
       </c>
       <c r="D7" s="23" t="n">
-        <v>46311</v>
+        <v>46303</v>
       </c>
       <c r="E7" s="24" t="inlineStr">
         <is>
@@ -15666,10 +15666,10 @@
         </is>
       </c>
       <c r="C8" s="22" t="n">
-        <v>46307</v>
+        <v>46299</v>
       </c>
       <c r="D8" s="23" t="n">
-        <v>46318</v>
+        <v>46310</v>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
@@ -15716,10 +15716,10 @@
         </is>
       </c>
       <c r="C9" s="22" t="n">
-        <v>46307</v>
+        <v>46299</v>
       </c>
       <c r="D9" s="23" t="n">
-        <v>46311</v>
+        <v>46303</v>
       </c>
       <c r="E9" s="24" t="inlineStr">
         <is>
@@ -15766,10 +15766,10 @@
         </is>
       </c>
       <c r="C10" s="22" t="n">
-        <v>46307</v>
+        <v>46299</v>
       </c>
       <c r="D10" s="23" t="n">
-        <v>46321</v>
+        <v>46313</v>
       </c>
       <c r="E10" s="24" t="inlineStr">
         <is>
@@ -15816,10 +15816,10 @@
         </is>
       </c>
       <c r="C11" s="22" t="n">
-        <v>46312</v>
+        <v>46304</v>
       </c>
       <c r="D11" s="23" t="n">
-        <v>46314</v>
+        <v>46306</v>
       </c>
       <c r="E11" s="24" t="inlineStr">
         <is>
@@ -15866,10 +15866,10 @@
         </is>
       </c>
       <c r="C12" s="22" t="n">
-        <v>46307</v>
+        <v>46299</v>
       </c>
       <c r="D12" s="23" t="n">
-        <v>46314</v>
+        <v>46306</v>
       </c>
       <c r="E12" s="24" t="inlineStr">
         <is>
@@ -15916,10 +15916,10 @@
         </is>
       </c>
       <c r="C13" s="22" t="n">
-        <v>46315</v>
+        <v>46307</v>
       </c>
       <c r="D13" s="23" t="n">
-        <v>46320</v>
+        <v>46312</v>
       </c>
       <c r="E13" s="24" t="inlineStr">
         <is>
@@ -15966,10 +15966,10 @@
         </is>
       </c>
       <c r="C14" s="22" t="n">
-        <v>46321</v>
+        <v>46313</v>
       </c>
       <c r="D14" s="23" t="n">
-        <v>46321</v>
+        <v>46313</v>
       </c>
       <c r="E14" s="24" t="inlineStr">
         <is>
@@ -16016,10 +16016,10 @@
         </is>
       </c>
       <c r="C15" s="22" t="n">
-        <v>46322</v>
+        <v>46314</v>
       </c>
       <c r="D15" s="23" t="n">
-        <v>46328</v>
+        <v>46320</v>
       </c>
       <c r="E15" s="24" t="inlineStr">
         <is>
@@ -16066,10 +16066,10 @@
         </is>
       </c>
       <c r="C16" s="22" t="n">
-        <v>46329</v>
+        <v>46321</v>
       </c>
       <c r="D16" s="23" t="n">
-        <v>46334</v>
+        <v>46326</v>
       </c>
       <c r="E16" s="24" t="inlineStr">
         <is>
@@ -16116,10 +16116,10 @@
         </is>
       </c>
       <c r="C17" s="22" t="n">
-        <v>46335</v>
+        <v>46327</v>
       </c>
       <c r="D17" s="23" t="n">
-        <v>46341</v>
+        <v>46333</v>
       </c>
       <c r="E17" s="24" t="inlineStr">
         <is>
@@ -16166,10 +16166,10 @@
         </is>
       </c>
       <c r="C18" s="22" t="n">
-        <v>46342</v>
+        <v>46334</v>
       </c>
       <c r="D18" s="23" t="n">
-        <v>46346</v>
+        <v>46338</v>
       </c>
       <c r="E18" s="24" t="inlineStr">
         <is>
@@ -22941,7 +22941,7 @@
       </c>
       <c r="C8" s="30" t="inlineStr">
         <is>
-          <t>De lunes a sábado: pretest del 20 al 25/10/2026 y postest del 03 al 08/11/2026. En lo posible, cada participante repite en el postest el mismo día de la semana del pretest.</t>
+          <t>De lunes a sábado: pretest del 12 al 17/10/2026 y postest del 26 al 31/10/2026. En lo posible, cada participante repite en el postest el mismo día de la semana del pretest.</t>
         </is>
       </c>
       <c r="D8" s="13" t="inlineStr">
@@ -31087,7 +31087,7 @@
       </c>
       <c r="H23" s="42" t="inlineStr">
         <is>
-          <t>Congelar la versión el 26/10/2026 y registrar su número; no publicar cambios entre el pretest y el postest</t>
+          <t>Congelar la versión el 18/10/2026 y registrar su número; no publicar cambios entre el pretest y el postest</t>
         </is>
       </c>
       <c r="I23" s="42" t="inlineStr">
@@ -31207,7 +31207,7 @@
       </c>
       <c r="H25" s="48" t="inlineStr">
         <is>
-          <t>Iniciar los trámites el 12/10/2026 y hacer seguimiento semanal con el asesor</t>
+          <t>Iniciar los trámites el 04/10/2026 y hacer seguimiento semanal con el asesor</t>
         </is>
       </c>
       <c r="I25" s="48" t="inlineStr">
@@ -38036,7 +38036,7 @@
       </c>
       <c r="D6" s="80" t="inlineStr">
         <is>
-          <t>Carta de presentación de la UDH emitida el 15/10/2026 y recibida por la Gerencia del diario el 16/10/2026.</t>
+          <t>Carta de presentación de la UDH emitida el 07/10/2026 y recibida por la Gerencia del diario el 08/10/2026.</t>
         </is>
       </c>
       <c r="E6" s="2" t="n"/>
@@ -38120,7 +38120,7 @@
       </c>
       <c r="D8" s="48" t="inlineStr">
         <is>
-          <t>Vigente de setiembre a diciembre de 2026; el campo termina el 20/11/2026.</t>
+          <t>Vigente de setiembre a diciembre de 2026; el campo termina el 12/11/2026.</t>
         </is>
       </c>
       <c r="E8" s="2" t="n"/>
@@ -38162,7 +38162,7 @@
       </c>
       <c r="D9" s="82" t="inlineStr">
         <is>
-          <t>Conformidad ética otorgada por el Comité de Ética de la UDH el 19/10/2026.</t>
+          <t>Conformidad ética otorgada por el Comité de Ética de la UDH el 11/10/2026.</t>
         </is>
       </c>
       <c r="E9" s="2" t="n"/>
@@ -38562,7 +38562,7 @@
       </c>
       <c r="D19" s="80" t="inlineStr">
         <is>
-          <t>Juicio de expertos concluido el 16/10/2026: V de Aiken SUS = 0.93; satisfacción = 0.91.</t>
+          <t>Juicio de expertos concluido el 08/10/2026: V de Aiken SUS = 0.93; satisfacción = 0.91.</t>
         </is>
       </c>
       <c r="E19" s="2" t="n"/>
@@ -38604,7 +38604,7 @@
       </c>
       <c r="D20" s="82" t="inlineStr">
         <is>
-          <t>Piloto con 20 lectores (17–19/10/2026): alfa SUS = 0.81; satisfacción = 0.86.</t>
+          <t>Piloto con 20 lectores (17–11/10/2026): alfa SUS = 0.81; satisfacción = 0.86.</t>
         </is>
       </c>
       <c r="E20" s="2" t="n"/>
@@ -38688,7 +38688,7 @@
       </c>
       <c r="D22" s="82" t="inlineStr">
         <is>
-          <t>Instrumentos cargados en el módulo del experimento el 19/10/2026.</t>
+          <t>Instrumentos cargados en el módulo del experimento el 11/10/2026.</t>
         </is>
       </c>
       <c r="E22" s="2" t="n"/>
@@ -38730,7 +38730,7 @@
       </c>
       <c r="D23" s="82" t="inlineStr">
         <is>
-          <t>Base de datos (tablas thesis_*) y contador de clics del portal instalados y probados el 19/10/2026.</t>
+          <t>Base de datos (tablas thesis_*) y contador de clics del portal instalados y probados el 11/10/2026.</t>
         </is>
       </c>
       <c r="E23" s="2" t="n"/>
@@ -38804,7 +38804,7 @@
       </c>
       <c r="D25" s="80" t="inlineStr">
         <is>
-          <t>PWA publicada; versión v1.3.2 para el pretest y v1.4.0 congelada el 26/10/2026.</t>
+          <t>PWA publicada; versión v1.3.2 para el pretest y v1.0.0-frozen-2026-10-18 congelada el 18/10/2026.</t>
         </is>
       </c>
       <c r="E25" s="2" t="n"/>
@@ -38846,7 +38846,7 @@
       </c>
       <c r="D26" s="82" t="inlineStr">
         <is>
-          <t>Pruebas técnicas documentadas (informe de pruebas, 18/10/2026).</t>
+          <t>Pruebas técnicas documentadas (informe de pruebas, 10/10/2026).</t>
         </is>
       </c>
       <c r="E26" s="2" t="n"/>
@@ -39046,7 +39046,7 @@
       </c>
       <c r="D31" s="80" t="inlineStr">
         <is>
-          <t>Cronograma aprobado por el asesor el 16/10/2026.</t>
+          <t>Cronograma aprobado por el asesor el 08/10/2026.</t>
         </is>
       </c>
       <c r="E31" s="2" t="n"/>
@@ -39172,7 +39172,7 @@
       </c>
       <c r="D34" s="82" t="inlineStr">
         <is>
-          <t>Copia cifrada implementada y probada (restauración de prueba el 18/10/2026).</t>
+          <t>Copia cifrada implementada y probada (restauración de prueba el 10/10/2026).</t>
         </is>
       </c>
       <c r="E34" s="2" t="n"/>
@@ -39214,7 +39214,7 @@
       </c>
       <c r="D35" s="82" t="inlineStr">
         <is>
-          <t>Matriz socializada con el asesor el 16/10/2026.</t>
+          <t>Matriz socializada con el asesor el 08/10/2026.</t>
         </is>
       </c>
       <c r="E35" s="2" t="n"/>
@@ -40056,7 +40056,7 @@
       </c>
       <c r="D56" s="82" t="inlineStr">
         <is>
-          <t>La autorización reemitida (23/10/2026) menciona expresamente el uso del contenido y la API del portal.</t>
+          <t>La autorización reemitida (15/10/2026) menciona expresamente el uso del contenido y la API del portal.</t>
         </is>
       </c>
       <c r="E56" s="2" t="n"/>

</xml_diff>